<commit_message>
Publish from Niche Template Studio
</commit_message>
<xml_diff>
--- a/free/Free-Freelance-Rate-Calculator.xlsx
+++ b/free/Free-Freelance-Rate-Calculator.xlsx
@@ -114,7 +114,7 @@
   </sheetPr>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="58" customWidth="1"/>
+    <col min="1" max="1" width="68" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="60" customWidth="1"/>
   </cols>
@@ -297,7 +297,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Created with AI assistance (AI-generated content); formulas recalculated and checked. A planning tool, not financial or tax advice.</t>
+          <t xml:space="preserve">Created with AI assistance (AI-generated content); formulas recalculated and checked in LibreOffice Calc. A planning tool, not financial or tax advice.</t>
         </is>
       </c>
     </row>

</xml_diff>